<commit_message>
tärkär gender, puk dictionary form
</commit_message>
<xml_diff>
--- a/data/morphemes.xlsx
+++ b/data/morphemes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sergeimalyshev/Desktop/Tocharian/Tocharian A/My grammar/Candrakanta/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{960C6D91-65E9-4E42-AE3B-0E0D18164D61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC64EAD6-D358-E148-BEBD-E2DF1BD7FC99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20" yWindow="580" windowWidth="29920" windowHeight="10340" activeTab="2" xr2:uid="{DFFD3512-190B-6C44-A03E-FE8C03207A6B}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8174" uniqueCount="3516">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8175" uniqueCount="3516">
   <si>
     <t>ID</t>
   </si>
@@ -58227,7 +58227,9 @@
       <c r="D1188" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="E1188" s="9"/>
+      <c r="E1188" s="9" t="s">
+        <v>2451</v>
+      </c>
       <c r="F1188" s="9"/>
       <c r="G1188" s="6" t="s">
         <v>2410</v>

</xml_diff>